<commit_message>
Updating with new Dev and Win profiles
</commit_message>
<xml_diff>
--- a/VaydeerMacropad.Mouse.VisualStudio.Template.xlsx
+++ b/VaydeerMacropad.Mouse.VisualStudio.Template.xlsx
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>C+5</t>
   </si>
@@ -462,17 +462,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -492,9 +486,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -577,22 +568,43 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
@@ -607,26 +619,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -665,7 +662,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F260F60A-DBEE-42CC-E5BD-D375680FC416}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{F260F60A-DBEE-42CC-E5BD-D375680FC416}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -721,7 +718,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAA941E0-F4D6-44EA-A8EB-038D50ADF789}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{CAA941E0-F4D6-44EA-A8EB-038D50ADF789}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -766,14 +763,14 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>34428</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>53800</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>68856</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>510745</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>530117</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>545173</xdr:rowOff>
     </xdr:to>
@@ -792,7 +789,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="34428" y="68856"/>
+          <a:off x="2207419" y="68856"/>
           <a:ext cx="476317" cy="476317"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -804,16 +801,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>77011</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>57636</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>64851</xdr:rowOff>
+      <xdr:rowOff>58395</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>579608</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>560233</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>561004</xdr:rowOff>
+      <xdr:rowOff>554548</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -830,7 +827,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3441160" y="64851"/>
+          <a:off x="1278128" y="58395"/>
           <a:ext cx="502597" cy="496153"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1374,223 +1371,229 @@
     <col min="4" max="4" width="4.85546875" customWidth="1"/>
     <col min="6" max="6" width="9.140625" customWidth="1"/>
     <col min="8" max="8" width="4.85546875" customWidth="1"/>
-    <col min="9" max="11" width="9.140625" style="33"/>
+    <col min="9" max="11" width="9.140625" style="30"/>
     <col min="12" max="12" width="4.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14"/>
-      <c r="B1" s="15"/>
-      <c r="C1" s="16"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="16"/>
+      <c r="A1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="13"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="13"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="13"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="17">
+      <c r="A2" s="14">
         <v>7</v>
       </c>
-      <c r="B2" s="18">
+      <c r="B2" s="15">
         <v>8</v>
       </c>
-      <c r="C2" s="19">
+      <c r="C2" s="16">
         <v>9</v>
       </c>
-      <c r="E2" s="17">
+      <c r="E2" s="14">
         <v>7</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="15">
         <v>8</v>
       </c>
-      <c r="G2" s="19">
+      <c r="G2" s="16">
         <v>9</v>
       </c>
-      <c r="M2" s="17">
+      <c r="M2" s="14">
         <v>7</v>
       </c>
-      <c r="N2" s="18">
+      <c r="N2" s="15">
         <v>8</v>
       </c>
-      <c r="O2" s="19">
+      <c r="O2" s="16">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="26" t="s">
+      <c r="A3" s="40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="47" t="s">
+      <c r="E3" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="45" t="s">
+      <c r="F3" s="42" t="s">
         <v>38</v>
       </c>
       <c r="G3" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="33" t="s">
+      <c r="I3" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="33" t="s">
+      <c r="K3" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="47" t="s">
+      <c r="M3" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="N3" s="55" t="s">
+      <c r="N3" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="O3" s="30" t="s">
+      <c r="O3" s="27" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="27" t="s">
+      <c r="A4" s="56"/>
+      <c r="B4" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="43"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="34" t="s">
+      <c r="E4" s="52"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="51"/>
+      <c r="M4" s="46"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="31" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="22">
+      <c r="A5" s="19">
         <v>4</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B5" s="18">
         <v>5</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="17">
         <v>6</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="19">
         <v>4</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="18">
         <v>5</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="17">
         <v>6</v>
       </c>
-      <c r="M5" s="22">
+      <c r="M5" s="19">
         <v>4</v>
       </c>
-      <c r="N5" s="21">
+      <c r="N5" s="18">
         <v>5</v>
       </c>
-      <c r="O5" s="20">
+      <c r="O5" s="17">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="E6" s="41" t="s">
+      <c r="C6" s="7"/>
+      <c r="E6" s="38" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="50" t="s">
+      <c r="F6" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="42" t="s">
+      <c r="G6" s="49" t="s">
         <v>33</v>
       </c>
-      <c r="M6" s="31" t="s">
+      <c r="M6" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="N6" s="32" t="s">
+      <c r="N6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="O6" s="42" t="s">
+      <c r="O6" s="49" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="E7" s="58" t="s">
+      <c r="C7" s="8"/>
+      <c r="E7" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="51"/>
-      <c r="G7" s="43"/>
-      <c r="M7" s="32" t="s">
+      <c r="F7" s="55"/>
+      <c r="G7" s="51"/>
+      <c r="M7" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="N7" s="32" t="s">
+      <c r="N7" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="O7" s="57"/>
+      <c r="O7" s="50"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="23">
+      <c r="A8" s="20">
         <v>1</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="21">
         <v>2</v>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="22">
         <v>3</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="20">
         <v>1</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="21">
         <v>2</v>
       </c>
-      <c r="G8" s="25">
+      <c r="G8" s="22">
         <v>3</v>
       </c>
-      <c r="M8" s="23">
+      <c r="M8" s="20">
         <v>1</v>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="21">
         <v>2</v>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="22">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="8"/>
-      <c r="E9" s="39" t="s">
+      <c r="A9" s="57" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="45" t="s">
+      <c r="B9" s="1"/>
+      <c r="C9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="G9" s="37" t="s">
+      <c r="G9" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="47" t="s">
+      <c r="M9" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="N9" s="45" t="s">
+      <c r="N9" s="42" t="s">
         <v>18</v>
       </c>
       <c r="O9" s="44" t="s">
@@ -1598,79 +1601,84 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="11"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="13"/>
-      <c r="E10" s="40" t="s">
+      <c r="A10" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="F10" s="46"/>
-      <c r="G10" s="38" t="s">
+      <c r="B10" s="9"/>
+      <c r="C10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="M10" s="52"/>
-      <c r="N10" s="46"/>
-      <c r="O10" s="53"/>
+      <c r="E10" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="43"/>
+      <c r="G10" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" s="41"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="45"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M11" s="35" t="s">
+      <c r="M11" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="N11" s="35" t="s">
+      <c r="N11" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="O11" s="36"/>
+      <c r="O11" s="33"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M12" s="36" t="s">
+      <c r="M12" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="N12" s="36" t="s">
+      <c r="N12" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="O12" s="36"/>
+      <c r="O12" s="33"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M13" s="35" t="s">
+      <c r="M13" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="N13" s="36"/>
-      <c r="O13" s="36"/>
+      <c r="N13" s="33"/>
+      <c r="O13" s="33"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M14" s="36" t="s">
+      <c r="M14" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="36" t="s">
+      <c r="N14" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="O14" s="36"/>
+      <c r="O14" s="33"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="M15" s="36" t="s">
+      <c r="M15" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="N15" s="36" t="s">
+      <c r="N15" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="O15" s="36"/>
+      <c r="O15" s="33"/>
     </row>
     <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="F6:F7"/>
     <mergeCell ref="M9:M10"/>
     <mergeCell ref="N9:N10"/>
     <mergeCell ref="O9:O10"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="O6:O7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="F6:F7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0" top="0.25" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>